<commit_message>
[TSR-264] roadmap: the pedido that queued forever against a backend that was up
Records what driving the real POS found that no harness could: a manual order
POST is preflighted (it carries Idempotency-Key), store-be's gateway did not
allow that header, and the POS cannot tell a blocked preflight from an unplugged
cable — so it retried a permanent failure as a temporary one, forever, with no
error surfaced at any layer.

Also records the end-to-end proof once the header was allowed: the queued pedido
replayed on its own into PM-000001, was walked to entregado through the UI, and
billed to consecutive …0241 ACCEPTED by Hacienda for a non-chain customer.

QA doc and its generated xlsx updated together, per the rule in CLAUDE.md: the
new rows say what to test and, for the CORS one, that curl cannot reproduce it
because curl does not preflight.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WER1ce22WMGh2NxvRi7pgm
</commit_message>
<xml_diff>
--- a/docs/qa/POS_FE_QA_ANALYSIS.xlsx
+++ b/docs/qa/POS_FE_QA_ANALYSIS.xlsx
@@ -52,7 +52,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Motor-Fiscal'!$A$1:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Catálogos-DataApi'!$A$1:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Código-Huérfano'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Verticales-TipoNegocio'!$A$1:$F$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Verticales-TipoNegocio'!$A$1:$F$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Hallazgos'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1023,10 +1023,10 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D37" s="2" t="n"/>
     </row>
@@ -4058,7 +4058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4215,12 +4215,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>TSR-151</t>
+          <t>TSR-151 · TSR-264</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Punto de entrega sin texto libre: registrado / receptor / cascada CR</t>
+          <t>Punto de entrega sin texto libre: registrado / receptor / cascada CR. La tarjeta mostraba la dirección del receptor sobre un payload que no la llevaba: probar con cliente SIN puntos registrados y cambiando de cliente con el modo ya en receptor</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4247,12 +4247,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>TSR-152</t>
+          <t>TSR-152 · TSR-264</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>El cuerpo del storefront (sin source) sigue validando igual — verificado</t>
+          <t>Idempotency-Key faltaba en el CORS del gateway: el preflight fallaba y el POS encolaba el pedido como si estuviera sin conexión, para siempre y sin error visible. Probar SIEMPRE desde el navegador — curl no hace preflight</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4264,12 +4264,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SelectField</t>
+          <t>Facturación de pedido manual (extremo a extremo)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Listbox propio, teclado + ARIA; 32 archivos convertidos sin tocar handlers</t>
+          <t>PM-000001 creado en el POS para cliente no-cadena, avanzado pendiente → procesando → enviado → entregado, facturado a consecutivo …0241 ACEPTADO</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -4279,29 +4279,29 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>TSR-153</t>
+          <t>TSR-264</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Un &lt;option&gt; nativo no se puede estilizar; el popup lo dibuja el SO</t>
+          <t>Facturar pedido sólo aparece en entregado; encabezado «Facturar pedido», cierre «Pedido facturado» / «Cerrar». invoice_sale_id queda escrito, así que no se puede facturar dos veces</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Menú 'Más' de pagos</t>
+          <t>Fechas de pedidos manuales</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Bug de capas CSS: .dropdown-menu fuera de @layer ganaba a las utilities</t>
+          <t>YYYY-MM-DD se leía como medianoche UTC → se mostraba un día antes en Costa Rica; el formateador estaba duplicado en dos páginas</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -4311,29 +4311,29 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>TSR-153</t>
+          <t>TSR-264</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Verificado en el CSS compilado</t>
+          <t>Los pedidos importados (DD/MM/YYYY) nunca tuvieron el fallo: sólo se ve en pedidos capturados en el POS. Verificar creación y entrega en lista y detalle</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Mesas / cuentas abiertas</t>
+          <t>SelectField</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Full-stack; una cuenta de bar es una mesa dinámica</t>
+          <t>Listbox propio, teclado + ARIA; 32 archivos convertidos sin tocar handlers</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -4343,12 +4343,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>TSR-154</t>
+          <t>TSR-153</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Direccionadas por branch_code entero (TSR-149)</t>
+          <t>Un &lt;option&gt; nativo no se puede estilizar; el popup lo dibuja el SO</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4360,12 +4360,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Combos</t>
+          <t>Menú 'Más' de pagos</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Explotan en componentes al agregar al carrito</t>
+          <t>Bug de capas CSS: .dropdown-menu fuera de @layer ganaba a las utilities</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -4375,12 +4375,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>TSR-154</t>
+          <t>TSR-153</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Un combo con 13% y exento no puede ser una línea plana en un comprobante fiscal</t>
+          <t>Verificado en el CSS compilado</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4392,12 +4392,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Servicio 10%</t>
+          <t>Mesas / cuentas abiertas</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Línea propia, nunca recargo sobre el total</t>
+          <t>Full-stack; una cuenta de bar es una mesa dinámica</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -4412,24 +4412,24 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Se excluye de su propia base o se compone en cada recálculo</t>
+          <t>Direccionadas por branch_code entero (TSR-149)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Cuenta dividida</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Por línea o en partes iguales; N documentos</t>
+          <t>Explotan en componentes al agregar al carrito</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>sharesReconcile verifica que las partes sumen la cuenta original</t>
+          <t>Un combo con 13% y exento no puede ser una línea plana en un comprobante fiscal</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4456,12 +4456,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Búsqueda por código</t>
+          <t>Servicio 10%</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Sin gate — cualquier organización</t>
+          <t>Línea propia, nunca recargo sobre el total</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -4471,12 +4471,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>TSR-155</t>
+          <t>TSR-154</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Verificado contra datos reales de dev; funciona sin conexión</t>
+          <t>Se excluye de su propia base o se compone en cada recálculo</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -4488,12 +4488,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Código de balanza</t>
+          <t>Cuenta dividida</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Peso/precio embebido en EAN-13, parametrizable</t>
+          <t>Por línea o en partes iguales; N documentos</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -4503,29 +4503,29 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>TSR-155</t>
+          <t>TSR-154</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>El layout no está estandarizado: cada tienda configura su balanza</t>
+          <t>sharesReconcile verifica que las partes sumen la cuenta original</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Proformas</t>
+          <t>Búsqueda por código</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Estado quote, no un tipo de documento</t>
+          <t>Sin gate — cualquier organización</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -4535,12 +4535,12 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>TSR-156</t>
+          <t>TSR-155</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Guarda bloquea quote → delivered: una cotización sin aprobar no debe facturarse</t>
+          <t>Verificado contra datos reales de dev; funciona sin conexión</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -4552,12 +4552,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Puntos de venta manuales</t>
+          <t>Código de balanza</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CRUD junto al importador de Excel</t>
+          <t>Peso/precio embebido en EAN-13, parametrizable</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -4567,12 +4567,12 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>TSR-157</t>
+          <t>TSR-155</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Totales derivados; sobre-asignar devuelve 422 nombrando la línea</t>
+          <t>El layout no está estandarizado: cada tienda configura su balanza</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -4584,12 +4584,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Happy hour</t>
+          <t>Proformas</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Ventanas que cruzan medianoche; nunca sube el precio</t>
+          <t>Estado quote, no un tipo de documento</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -4599,12 +4599,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>TSR-158</t>
+          <t>TSR-156</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>El servidor re-resuelve al enviar: el reloj del cliente no fija precios fiscales</t>
+          <t>Guarda bloquea quote → delivered: una cotización sin aprobar no debe facturarse</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -4616,12 +4616,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Lotes / FEFO</t>
+          <t>Puntos de venta manuales</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Primero el que vence, no el que llegó</t>
+          <t>CRUD junto al importador de Excel</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -4631,12 +4631,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>TSR-159</t>
+          <t>TSR-157</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Stock sin fecha va al final; 0 días = vence hoy</t>
+          <t>Totales derivados; sobre-asignar devuelve 422 nombrando la línea</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -4648,12 +4648,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Facturación recurrente</t>
+          <t>Happy hour</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Cadencia con recorte de mes</t>
+          <t>Ventanas que cruzan medianoche; nunca sube el precio</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -4663,29 +4663,29 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>TSR-160</t>
+          <t>TSR-158</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Genera borrador, nunca transmite; falta EventBridge</t>
+          <t>El servidor re-resuelve al enviar: el reloj del cliente no fija precios fiscales</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Unidades con conversión</t>
+          <t>Lotes / FEFO</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Stock en rollos, venta por metro</t>
+          <t>Primero el que vence, no el que llegó</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -4695,29 +4695,29 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>TSR-161</t>
+          <t>TSR-159</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Factor 0 rechazado; price_override gana</t>
+          <t>Stock sin fecha va al final; 0 días = vence hoy</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Agenda</t>
+          <t>Facturación recurrente</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Un módulo, dos verticales (salón y taller)</t>
+          <t>Cadencia con recorte de mes</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -4727,12 +4727,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>TSR-162</t>
+          <t>TSR-160</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>asset_id nullable: el salón agenda una persona, el taller persona + vehículo</t>
+          <t>Genera borrador, nunca transmite; falta EventBridge</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -4744,12 +4744,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Órdenes de trabajo</t>
+          <t>Unidades con conversión</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>PM con order_type='work_order'</t>
+          <t>Stock en rollos, venta por metro</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -4759,29 +4759,29 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>TSR-163</t>
+          <t>TSR-161</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>No es una entidad nueva; client_assets sí, para historial por activo</t>
+          <t>Factor 0 rechazado; price_override gana</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Importación Excel estructurada</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Descuento 07 Comercial + impuestos del producto</t>
+          <t>Un módulo, dos verticales (salón y taller)</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -4791,29 +4791,29 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>TSR-152</t>
+          <t>TSR-162</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Sólo 01/03 desvían IVA a fábrica; 07 debe seguir siendo rebaja de precio</t>
+          <t>asset_id nullable: el salón agenda una persona, el taller persona + vehículo</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Ticket 80 mm</t>
+          <t>Órdenes de trabajo</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Generado en el backend (ticket.html → wkhtmltopdf → S3)</t>
+          <t>PM con order_type='work_order'</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -4823,12 +4823,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>TSR-127</t>
+          <t>TSR-163</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Se descartó imprimir en el navegador: dos maquetadores harían que una reimpresión no coincida con el original</t>
+          <t>No es una entidad nueva; client_assets sí, para historial por activo</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -4840,37 +4840,101 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Importación Excel estructurada</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Descuento 07 Comercial + impuestos del producto</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>TSR-152</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Sólo 01/03 desvían IVA a fábrica; 07 debe seguir siendo rebaja de precio</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Ticket 80 mm</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Generado en el backend (ticket.html → wkhtmltopdf → S3)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>TSR-127</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Se descartó imprimir en el navegador: dos maquetadores harían que una reimpresión no coincida con el original</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>Ferias</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Fuera del selector a propósito</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>❌ Faltante</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>TSR-164</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Es agrupación multi-organización, no un tipo de negocio</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F25"/>
+  <autoFilter ref="A1:F27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record TSR-327..334 — consecutives, multi-role, live permissions, document detail and flow order
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/POS_FE_QA_ANALYSIS.xlsx
+++ b/docs/qa/POS_FE_QA_ANALYSIS.xlsx
@@ -42,8 +42,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Pedidos'!$A$1:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Confirmaciones'!$A$1:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Reportes'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Sesiones-Puestos'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Roles-RBAC'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Sesiones-Puestos'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Roles-RBAC'!$A$1:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Config-Organización'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'CMS-Storefront'!$A$1:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Programas'!$A$1:$F$2</definedName>
@@ -86,7 +86,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -120,6 +120,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
@@ -136,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -163,10 +168,13 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -534,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -713,121 +721,121 @@
       <c r="D14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>⏸️ Deshabilitado</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Implementado, pero apagado a propósito con un flag del producto hasta completarlo</t>
+        </is>
+      </c>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Hojas por módulo</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Funcionalidades</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Alta prioridad</t>
         </is>
-      </c>
-      <c r="D16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Autenticación</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>4</v>
       </c>
       <c r="D17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Autenticación</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>POS-Documentos</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Facturación-Hacienda</t>
+          <t>POS-Documentos</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Productos</t>
+          <t>Facturación-Hacienda</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Categorías</t>
+          <t>Productos</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="D22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Clientes-B2B</t>
+          <t>Categorías</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C23" s="2" t="n">
         <v>0</v>
@@ -837,119 +845,119 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Pedidos</t>
+          <t>Clientes-B2B</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Confirmaciones</t>
+          <t>Pedidos</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Reportes</t>
+          <t>Confirmaciones</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Sesiones-Puestos</t>
+          <t>Reportes</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Roles-RBAC</t>
+          <t>Sesiones-Puestos</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Config-Organización</t>
+          <t>Roles-RBAC</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CMS-Storefront</t>
+          <t>Config-Organización</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Programas</t>
+          <t>CMS-Storefront</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Perfil</t>
+          <t>Programas</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -963,147 +971,139 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Shell-Transversales</t>
+          <t>Perfil</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Motor-Fiscal</t>
+          <t>Shell-Transversales</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Catálogos-DataApi</t>
+          <t>Motor-Fiscal</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Código-Huérfano</t>
+          <t>Catálogos-DataApi</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>Código-Huérfano</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>Verticales-TipoNegocio</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B38" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="C37" s="2" t="n">
+      <c r="C38" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D37" s="2" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
       <c r="D38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Riesgos críticos (roadmap §6) que QA debe conocer</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="n"/>
       <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="n"/>
       <c r="D39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Riesgos críticos (roadmap §6) que QA debe conocer</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>TSR</t>
         </is>
       </c>
-      <c r="D40" s="10" t="inlineStr">
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>Severidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Credenciales fiscales (P12, PIN, ATV) en texto plano en Postgres y retornadas por GET; realm OAuth hardcodeado a staging</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>TSR-002, TSR-003</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Crítica (legal)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Verdad fiscal duplicada: dos asignadores de consecutivo, tres motores de impuestos sincronizados 'por convención'</t>
+          <t>Credenciales fiscales (P12, PIN, ATV) en texto plano en Postgres y retornadas por GET; realm OAuth hardcodeado a staging</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>TSR-004</t>
+          <t>TSR-002, TSR-003</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1115,42 +1115,64 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Gateway de markets-api no valida userId↔sub; el RBAC confía en una validación inexistente</t>
+          <t>Verdad fiscal duplicada: dos asignadores de consecutivo, tres motores de impuestos sincronizados 'por convención'</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>TSR-029</t>
+          <t>TSR-004</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Crítica (seguridad)</t>
+          <t>Crítica (legal)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Gateway de markets-api no valida userId↔sub; el RBAC confía en una validación inexistente</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>TSR-029</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Crítica (seguridad)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Servicios Python (sales/orders/data-api) sin checks de membresía; docs fiscales y credenciales ATV expuestos</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>TSR-030, TSR-031</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Crítica (seguridad)</t>
         </is>
@@ -1179,32 +1201,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -1426,32 +1448,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -1533,7 +1555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1545,32 +1567,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -1619,61 +1641,157 @@
           <t>PuestosPage, catálogo de tipos de sucursal</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>🟡 Parcial</t>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TSR-139</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>useBranchTypes con TODO — catálogo en proceso en cross-app-be</t>
+          <t>Catálogo branch_types implementado en store-be (4 rutas); las sucursales se direccionan por code entero, no UUID (TSR-149)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Detalle de terminal</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>TerminalDetailPage: datos, consecutivo por tipo de documento (último número + próximo consecutivo) y documentos emitidos</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>TSR-327, TSR-328</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Tarjetas gateadas por admin:consecutives:read y documents:emitted:read</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Consecutivos (Administración interna)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ConsecutivesPage: filtros sucursal → terminal → tipo de documento con el DSL search=, persistidos en la URL</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>TSR-327, TSR-329</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Verificar que el filtro sobrevive a recargar y que cambiar de sucursal limpia la terminal</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Ajuste manual de consecutivo</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Drawer en dos pasos con confirmación y acuse; el BE solo permite subir el número, con bloqueo de fila y bitácora</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>TSR-327</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Sensible fiscal: número menor → error; venta concurrente → 409; sin admin:consecutives:update → 403 y botón oculto</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Aprobación de cierres</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Autorización de cierre de caja</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>🔒 Bloqueado por backend</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>TSR-010</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>is_manager default True en BE — cualquier usuario aprueba cierres</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
+  <autoFilter ref="A1:F7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1684,7 +1802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1696,32 +1814,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -1735,7 +1853,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Invitar, asignar rol, remover</t>
+          <t>Invitar, asignar roles (varios por miembro), quitar roles, remover</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -1745,12 +1863,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TSR-024</t>
+          <t>TSR-024, TSR-330</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Al menos un rol por miembro; el último propietario conserva owner; nadie edita sus propios roles</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1762,12 +1880,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Roles y matriz de permisos</t>
+          <t>Cambio de rol en sesión</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>RolesPage + RoleDrawerForm + PermissionMatrix org-scoped; catálogo espejo 1:1 del sidebar</t>
+          <t>Perfil → Rol en esta organización: elegir el rol activo sin cerrar sesión</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -1777,12 +1895,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TSR-037</t>
+          <t>TSR-330</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Permisos del rol activo, nunca la unión</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1794,37 +1912,101 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Cambios de permisos en vivo</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Cambios de rol/permisos llegan por AppSync al POS abierto</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>TSR-331</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Requiere la política IAM de management-be; probar con dos sesiones</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Roles y matriz de permisos</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>RolesPage + RoleDrawerForm + PermissionMatrix org-scoped; catálogo espejo 1:1 del sidebar</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>TSR-037</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>Gating de acciones app-wide</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>133 elementos gateados (hide-not-disable) + nav + doc-types + org-settings por tarjeta</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>✅ Completo</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>TSR-110, TSR-038, TSR-109, TSR-107</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>usePermissions() fail-open mientras RBAC_ENFORCEMENT=log — no confiable hasta el flip (TSR-027)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>TSR-110, TSR-038, TSR-109, TSR-107, TSR-332</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>usePermissions() fail-closed (2026-09-22); sidebar desde módulos disponibles; agregar→create, editar→update, estado/eliminar→delete. BE aún en RBAC_ENFORCEMENT=log (TSR-027)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1847,32 +2029,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -1998,32 +2180,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -2213,32 +2395,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -2300,32 +2482,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -2387,32 +2569,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -2826,32 +3008,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -3361,32 +3543,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -3640,32 +3822,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -3951,32 +4133,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -4102,32 +4284,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -4432,24 +4614,24 @@
           <t>Full-stack; una cuenta de bar es una mesa dinámica</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>✅ Completo</t>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>⏸️ Deshabilitado</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>TSR-154</t>
+          <t>TSR-154, TSR-333</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Direccionadas por branch_code entero (TSR-149)</t>
+          <t>Pestaña Mesas deshabilitada en el POS integrado (POS_TABLES_ENABLED = false) hasta que existan las pantallas de administración</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
     </row>
@@ -4987,22 +5169,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>TSR</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Hallazgo</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Detalle / evidencia</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Severidad</t>
         </is>
@@ -5516,32 +5698,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -5667,32 +5849,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -6106,32 +6288,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -6353,32 +6535,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -6504,32 +6686,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -6591,32 +6773,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>
@@ -6742,32 +6924,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Funcionalidad</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Incidencia (TSR)</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Bugs / Riesgos</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Prioridad QA</t>
         </is>

</xml_diff>

<commit_message>
docs: TSR-125/335..343 — import, other charges, early-payment NC, two decimals; dev migrations applied
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/POS_FE_QA_ANALYSIS.xlsx
+++ b/docs/qa/POS_FE_QA_ANALYSIS.xlsx
@@ -49,7 +49,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Programas'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Perfil'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Shell-Transversales'!$A$1:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Motor-Fiscal'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Motor-Fiscal'!$A$1:$F$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Catálogos-DataApi'!$A$1:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Código-Huérfano'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Verticales-TipoNegocio'!$A$1:$F$27</definedName>
@@ -1003,10 +1003,10 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D35" s="2" t="n"/>
     </row>
@@ -2996,7 +2996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3399,22 +3399,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Bloque OtherCharges v4.4 (códigos 01–10/99, hasta 15/doc; 04 exige tercero)</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>❌ Faltante</t>
+          <t>Bloque OtrosCargos v4.4 (01–10/99, hasta 15/doc; 04 exige id + nombre del tercero; 99 exige naturaleza); sección en el checkout; 10% de servicio = código 06</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>TSR-125</t>
+          <t>TSR-125, TSR-337</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>No implementado en FE ni en BE de ventas; useAllOtherCharges sin usar</t>
+          <t>Resuelto 2026-09-23. Probar porcentaje vs monto fijo; 04 sin tercero y 99 sin naturaleza bloquean; el total a pagar incluye los cargos; detalle y PDF listan cada cargo</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3426,12 +3426,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Referencias</t>
+          <t>Importar XML de Hacienda</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ReferencesSection en todos los documentos; obligatoria en NC/ND/REP y FE con exoneración local; restricciones por tipo de documento aplicadas</t>
+          <t>Uno o varios XML firmados (v4.3/v4.4) desde Documentos o Históricos; barra por archivo + % total; resultado por la campana</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -3441,12 +3441,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>TSR-126</t>
+          <t>TSR-335, TSR-336</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>El enum del BE estaba mal en 8 de 14 códigos (06 es Devolución de mercancía, no sustitución por contingencia) y rechazaba el 17. Probar: sustituir un comprobante provisional/de contingencia desde una Factura; other_type/other_code con 99; Razon obligatoria; tope de 10; que el desplegable no ofrezca 17 fuera de REP ni 16 fuera de FEC</t>
+          <t>Probar con be/sales-be/xml-docs/: producción → No pertenece a este ambiente; XML ajeno → no pertenece a la organización; duplicado; no-XML ignorado; etiqueta Importado en la lista</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3458,27 +3458,27 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Suma de medios de pago</t>
+          <t>Descuento por pronto pago</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Regla Σ MedioPago == TotalComprobante</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>🔒 Bloqueado por backend</t>
+          <t>NC financiera (referencia 09) desde la factura aceptada o el pedido facturado; monto con IVA incluido + tarifa del original</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TSR-340, TSR-341</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>No se valida en el BE de ventas (CALCULATION_AUDIT §4) — probar pagos que no cuadran</t>
+          <t>IVA se rebaja del monto; monto &gt; saldo bloquea; documentos relacionados enlazados; Monto final baja al aceptarse la NC; el pedido lista la nota</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -3490,37 +3490,101 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Referencias</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ReferencesSection en todos los documentos; obligatoria en NC/ND/REP y FE con exoneración local; restricciones por tipo de documento aplicadas</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>TSR-126</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>El enum del BE estaba mal en 8 de 14 códigos (06 es Devolución de mercancía, no sustitución por contingencia) y rechazaba el 17. Probar: sustituir un comprobante provisional/de contingencia desde una Factura; other_type/other_code con 99; Razon obligatoria; tope de 10; que el desplegable no ofrezca 17 fuera de REP ni 16 fuera de FEC</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Suma de medios de pago</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Regla Σ MedioPago == TotalComprobante</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>🔒 Bloqueado por backend</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>No se valida en el BE de ventas (CALCULATION_AUDIT §4) — probar pagos que no cuadran</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Redondeo</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Decimal(18,5), round-half-up en el 6º dígito según spec</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>⚠️ Sin verificar</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>TSR-004</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>FE opera en float de JS; verificar contra totales del BE</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Dos decimales por línea (ROUND_HALF_UP) en FE y BE; totales = suma de líneas redondeadas</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>✅ Completo</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>TSR-004, TSR-343</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Cambiado 2026-09-23. Probar precio con &gt;2 decimales y exoneración 50% (563.29 → 281.65 / 281.64) contra el XML firmado</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:F18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4085,7 +4149,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>useAllOtherCharges (TSR-125), useAllDocumentTypes, PharmaceuticalForms, Regimes, NationalTaxpayerCompanies, NotificationCodes, Transactions, TaxConditions, TaxRateCodes, useDollarRate/useEuroRate</t>
+          <t>useAllDocumentTypes, PharmaceuticalForms, Regimes, NationalTaxpayerCompanies, NotificationCodes, Transactions, TaxConditions, TaxRateCodes, useDollarRate/useEuroRate</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -5330,12 +5394,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Otros cargos (documento) no implementado</t>
+          <t>Otros cargos (documento) — RESUELTO 2026-09-23</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bloque OtherCharges v4.4 (códigos 01–10/99, hasta 15/doc) ausente en FE y en el BE de ventas; useAllOtherCharges sin usar; además Σ MedioPago == TotalComprobante no se valida en BE</t>
+          <t>Sección en el checkout con el catálogo, reglas iguales al BE, total a pagar = carrito + cargos, 10% de servicio como código 06; el BE usaba nombres de elemento v4.3 (TSR-337), corregidos</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">

</xml_diff>